<commit_message>
Data room revised to the demo critic: cash reconciles, ordinary ids, decoys with teeth, seeded noise, a clean room, a sealed-variant switch
</commit_message>
<xml_diff>
--- a/data_room/hollis_voice/02_financials/cap_table.xlsx
+++ b/data_room/hollis_voice/02_financials/cap_table.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Cap_Table" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="CAP_TOTAL_PCT">Cap_Table!$D$12</definedName>
+    <definedName name="CAP_TOTAL_PCT">Cap_Table!$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
   <si>
     <t>Hollis Voice, Inc.: fully diluted cap table</t>
   </si>
@@ -70,7 +70,10 @@
     <t>Preferred (from SAFE)</t>
   </si>
   <si>
-    <t>Anselm Hartley (angel) (SAFE converted)</t>
+    <t>Winifred Hartley (angel) (SAFE converted)</t>
+  </si>
+  <si>
+    <t>Ostrander Lane Ventures II, LP (SAFE converted)</t>
   </si>
   <si>
     <t>Series A investors (new)</t>
@@ -103,7 +106,10 @@
     <t>Tidewater Seed Fund I, LP</t>
   </si>
   <si>
-    <t>Anselm Hartley (angel)</t>
+    <t>Winifred Hartley (angel)</t>
+  </si>
+  <si>
+    <t>Ostrander Lane Ventures II, LP</t>
   </si>
   <si>
     <t>Total SAFEs</t>
@@ -524,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -570,19 +576,19 @@
         <v>9</v>
       </c>
       <c r="C5" s="4">
-        <v>4400000</v>
+        <v>4437000</v>
       </c>
       <c r="D5" s="5">
-        <f>C5/C$12</f>
-        <v>0.36666666666666664</v>
+        <f>C5/C$13</f>
+        <v>0.30761231281198004</v>
       </c>
       <c r="E5" s="4">
         <f>C5</f>
-        <v>4400000</v>
+        <v>4437000</v>
       </c>
       <c r="F5" s="5">
-        <f>E5/E$12</f>
-        <v>0.3055555555555556</v>
+        <f>E5/E$13</f>
+        <v>0.25634359400998336</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -593,19 +599,19 @@
         <v>9</v>
       </c>
       <c r="C6" s="4">
-        <v>3600000</v>
+        <v>3598000</v>
       </c>
       <c r="D6" s="5">
-        <f>C6/C$12</f>
-        <v>0.3</v>
+        <f>C6/C$13</f>
+        <v>0.24944536882972823</v>
       </c>
       <c r="E6" s="4">
         <f>C6</f>
-        <v>3600000</v>
+        <v>3598000</v>
       </c>
       <c r="F6" s="5">
-        <f>E6/E$12</f>
-        <v>0.25</v>
+        <f>E6/E$13</f>
+        <v>0.2078711406914402</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -616,19 +622,19 @@
         <v>12</v>
       </c>
       <c r="C7" s="4">
-        <v>1150000</v>
+        <v>1148000</v>
       </c>
       <c r="D7" s="5">
-        <f>C7/C$12</f>
-        <v>0.09583333333333334</v>
+        <f>C7/C$13</f>
+        <v>0.07958957293399889</v>
       </c>
       <c r="E7" s="4">
         <f>C7</f>
-        <v>1150000</v>
+        <v>1148000</v>
       </c>
       <c r="F7" s="5">
-        <f>E7/E$12</f>
-        <v>0.0798611111111111</v>
+        <f>E7/E$13</f>
+        <v>0.06632464411166575</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -639,19 +645,19 @@
         <v>14</v>
       </c>
       <c r="C8" s="4">
-        <v>850000</v>
+        <v>1034000</v>
       </c>
       <c r="D8" s="5">
-        <f>C8/C$12</f>
-        <v>0.07083333333333333</v>
+        <f>C8/C$13</f>
+        <v>0.07168607875762618</v>
       </c>
       <c r="E8" s="4">
         <f>C8</f>
-        <v>850000</v>
+        <v>1034000</v>
       </c>
       <c r="F8" s="5">
-        <f>E8/E$12</f>
-        <v>0.059027777777777776</v>
+        <f>E8/E$13</f>
+        <v>0.05973839896468848</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -662,18 +668,18 @@
         <v>16</v>
       </c>
       <c r="C9" s="4">
-        <v>1200000</v>
+        <v>1442400</v>
       </c>
       <c r="D9" s="5">
-        <f>C9/C$12</f>
+        <f>C9/C$13</f>
         <v>0.1</v>
       </c>
       <c r="E9" s="4">
         <f>C9</f>
-        <v>1200000</v>
+        <v>1442400</v>
       </c>
       <c r="F9" s="5">
-        <f>E9/E$12</f>
+        <f>E9/E$13</f>
         <v>0.08333333333333333</v>
       </c>
     </row>
@@ -685,18 +691,18 @@
         <v>16</v>
       </c>
       <c r="C10" s="4">
-        <v>800000</v>
+        <v>961600</v>
       </c>
       <c r="D10" s="5">
-        <f>C10/C$12</f>
+        <f>C10/C$13</f>
         <v>0.06666666666666667</v>
       </c>
       <c r="E10" s="4">
         <f>C10</f>
-        <v>800000</v>
+        <v>961600</v>
       </c>
       <c r="F10" s="5">
-        <f>E10/E$12</f>
+        <f>E10/E$13</f>
         <v>0.05555555555555555</v>
       </c>
     </row>
@@ -705,91 +711,91 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4">
+        <v>1803000</v>
+      </c>
+      <c r="D11" s="5">
+        <f>C11/C$13</f>
+        <v>0.125</v>
+      </c>
+      <c r="E11" s="4">
+        <f>C11</f>
+        <v>1803000</v>
+      </c>
+      <c r="F11" s="5">
+        <f>E11/E$13</f>
+        <v>0.10416666666666667</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="4">
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="4">
         <v>0</v>
       </c>
-      <c r="D11" s="5">
-        <f>C11/C$12</f>
+      <c r="D12" s="5">
+        <f>C12/C$13</f>
         <v>0</v>
       </c>
-      <c r="E11" s="4">
-        <f>B25</f>
-        <v>2400000</v>
-      </c>
-      <c r="F11" s="5">
-        <f>E11/E$12</f>
+      <c r="E12" s="4">
+        <f>B27</f>
+        <v>2884800</v>
+      </c>
+      <c r="F12" s="5">
+        <f>E12/E$13</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="7">
-        <f>SUM(C5:C11)</f>
-        <v>12000000</v>
-      </c>
-      <c r="D12" s="8">
-        <f>SUM(D5:D11)</f>
+    <row r="13" spans="1:6">
+      <c r="A13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="7">
+        <f>SUM(C5:C12)</f>
+        <v>14424000</v>
+      </c>
+      <c r="D13" s="8">
+        <f>SUM(D5:D12)</f>
         <v>1.0</v>
       </c>
-      <c r="E12" s="7">
-        <f>SUM(E5:E11)</f>
-        <v>14400000</v>
-      </c>
-      <c r="F12" s="8">
-        <f>SUM(F5:F11)</f>
+      <c r="E13" s="7">
+        <f>SUM(E5:E12)</f>
+        <v>17308800</v>
+      </c>
+      <c r="F13" s="8">
+        <f>SUM(F5:F12)</f>
         <v>1.0</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="3" t="s">
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="E16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="4">
-        <v>1200000</v>
-      </c>
-      <c r="C16" s="4">
-        <v>12000000</v>
-      </c>
-      <c r="D16" s="5">
-        <f>B16/C16</f>
-        <v>0.1</v>
-      </c>
-      <c r="E16" s="9">
-        <f>C16/C$12</f>
-        <v>1.0</v>
-      </c>
-      <c r="F16" s="4">
-        <f>B16/E16</f>
-        <v>1200000.0</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -797,60 +803,90 @@
         <v>28</v>
       </c>
       <c r="B17" s="4">
-        <v>800000</v>
+        <v>1200000</v>
       </c>
       <c r="C17" s="4">
         <v>12000000</v>
       </c>
       <c r="D17" s="5">
         <f>B17/C17</f>
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="9">
+        <f>C17/C$13</f>
+        <v>0.831946755407654</v>
+      </c>
+      <c r="F17" s="4">
+        <f>ROUND(B17/E17,0)</f>
+        <v>1442400</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="4">
+        <v>800000</v>
+      </c>
+      <c r="C18" s="4">
+        <v>12000000</v>
+      </c>
+      <c r="D18" s="5">
+        <f>B18/C18</f>
         <v>0.06666666666666667</v>
       </c>
-      <c r="E17" s="9">
-        <f>C17/C$12</f>
-        <v>1.0</v>
-      </c>
-      <c r="F17" s="4">
-        <f>B17/E17</f>
-        <v>800000.0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="7">
-        <f>SUM(B16:B17)</f>
-        <v>2000000</v>
-      </c>
-      <c r="D18" s="8">
-        <f>SUM(D16:D17)</f>
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="F18" s="7">
-        <f>SUM(F16:F17)</f>
-        <v>2000000.0</v>
+      <c r="E18" s="9">
+        <f>C18/C$13</f>
+        <v>0.831946755407654</v>
+      </c>
+      <c r="F18" s="4">
+        <f>ROUND(B18/E18,0)</f>
+        <v>961600</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="4">
+        <v>3500000</v>
+      </c>
+      <c r="C19" s="4">
+        <v>28000000</v>
+      </c>
+      <c r="D19" s="5">
+        <f>B19/C19</f>
+        <v>0.125</v>
+      </c>
+      <c r="E19" s="9">
+        <f>C19/C$13</f>
+        <v>1.9412090959511925</v>
+      </c>
+      <c r="F19" s="4">
+        <f>ROUND(B19/E19,0)</f>
+        <v>1803000</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="4">
-        <v>45000000</v>
+      <c r="B20" s="7">
+        <f>SUM(B17:B19)</f>
+        <v>5500000</v>
+      </c>
+      <c r="D20" s="8">
+        <f>SUM(D17:D19)</f>
+        <v>0.2916666666666667</v>
+      </c>
+      <c r="F20" s="7">
+        <f>SUM(F17:F19)</f>
+        <v>4207000</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" t="s">
+      <c r="A22" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="B22" s="4">
-        <v>9000000</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -858,17 +894,15 @@
         <v>33</v>
       </c>
       <c r="B23" s="4">
-        <f>B21+B22</f>
-        <v>54000000</v>
+        <v>45000000</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="9">
-        <f>B21/C12</f>
-        <v>3.75</v>
+      <c r="B24" s="4">
+        <v>9000000</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -876,22 +910,40 @@
         <v>35</v>
       </c>
       <c r="B25" s="4">
-        <f>B22/B24</f>
-        <v>2400000</v>
+        <f>B23+B24</f>
+        <v>54000000</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="5">
-        <f>B22/B23</f>
+      <c r="B26" s="9">
+        <f>B23/C13</f>
+        <v>3.119800332778702</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="4">
+        <f>B24/B26</f>
+        <v>2884800</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="5">
+        <f>B24/B25</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="2" t="s">
-        <v>37</v>
+    <row r="31" spans="1:6">
+      <c r="A31" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>